<commit_message>
feat: carga de aplicación
</commit_message>
<xml_diff>
--- a/app/ComisionesCalculadas.xlsx
+++ b/app/ComisionesCalculadas.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,62 +417,62 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>empleado_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Nombre y Apellido</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Comisión</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>tip_documento</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>num_documento</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>nom_empleado</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ape_empleado</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>cod_cargo</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>cod_departamento</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>mnt_salario</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>mnt_tope_comision</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>comision_calculada</t>
         </is>
@@ -538,10 +526,8 @@
       <c r="K2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -592,10 +578,8 @@
       <c r="K3" t="n">
         <v>300</v>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
+      <c r="L3" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="4">
@@ -646,10 +630,8 @@
       <c r="K4" t="n">
         <v>0</v>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -700,10 +682,8 @@
       <c r="K5" t="n">
         <v>0</v>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -754,10 +734,8 @@
       <c r="K6" t="n">
         <v>550</v>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>550</t>
-        </is>
+      <c r="L6" t="n">
+        <v>550</v>
       </c>
     </row>
     <row r="7">
@@ -808,10 +786,8 @@
       <c r="K7" t="n">
         <v>0</v>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -862,10 +838,8 @@
       <c r="K8" t="n">
         <v>0</v>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -916,10 +890,8 @@
       <c r="K9" t="n">
         <v>310</v>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>310</t>
-        </is>
+      <c r="L9" t="n">
+        <v>310</v>
       </c>
     </row>
     <row r="10">
@@ -970,10 +942,8 @@
       <c r="K10" t="n">
         <v>0</v>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1024,10 +994,8 @@
       <c r="K11" t="n">
         <v>520</v>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>520</t>
-        </is>
+      <c r="L11" t="n">
+        <v>520</v>
       </c>
     </row>
     <row r="12">
@@ -1078,10 +1046,8 @@
       <c r="K12" t="n">
         <v>0</v>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1132,10 +1098,8 @@
       <c r="K13" t="n">
         <v>0</v>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1186,10 +1150,8 @@
       <c r="K14" t="n">
         <v>330</v>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>330</t>
-        </is>
+      <c r="L14" t="n">
+        <v>330</v>
       </c>
     </row>
     <row r="15">
@@ -1240,10 +1202,8 @@
       <c r="K15" t="n">
         <v>0</v>
       </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1294,10 +1254,8 @@
       <c r="K16" t="n">
         <v>570</v>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>570</t>
-        </is>
+      <c r="L16" t="n">
+        <v>570</v>
       </c>
     </row>
     <row r="17">
@@ -1348,10 +1306,8 @@
       <c r="K17" t="n">
         <v>0</v>
       </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L17" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1402,10 +1358,8 @@
       <c r="K18" t="n">
         <v>0</v>
       </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1456,10 +1410,8 @@
       <c r="K19" t="n">
         <v>305</v>
       </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>305</t>
-        </is>
+      <c r="L19" t="n">
+        <v>305</v>
       </c>
     </row>
     <row r="20">
@@ -1510,10 +1462,8 @@
       <c r="K20" t="n">
         <v>0</v>
       </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1564,10 +1514,8 @@
       <c r="K21" t="n">
         <v>530</v>
       </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>530</t>
-        </is>
+      <c r="L21" t="n">
+        <v>530</v>
       </c>
     </row>
     <row r="22">
@@ -1618,10 +1566,8 @@
       <c r="K22" t="n">
         <v>0</v>
       </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1672,10 +1618,8 @@
       <c r="K23" t="n">
         <v>0</v>
       </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1726,10 +1670,8 @@
       <c r="K24" t="n">
         <v>325</v>
       </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>325</t>
-        </is>
+      <c r="L24" t="n">
+        <v>325</v>
       </c>
     </row>
     <row r="25">
@@ -1780,10 +1722,8 @@
       <c r="K25" t="n">
         <v>0</v>
       </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1834,10 +1774,8 @@
       <c r="K26" t="n">
         <v>560</v>
       </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>560</t>
-        </is>
+      <c r="L26" t="n">
+        <v>560</v>
       </c>
     </row>
     <row r="27">
@@ -1888,10 +1826,8 @@
       <c r="K27" t="n">
         <v>0</v>
       </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1942,10 +1878,8 @@
       <c r="K28" t="n">
         <v>0</v>
       </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -1996,10 +1930,8 @@
       <c r="K29" t="n">
         <v>315</v>
       </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>315</t>
-        </is>
+      <c r="L29" t="n">
+        <v>315</v>
       </c>
     </row>
     <row r="30">
@@ -2050,10 +1982,8 @@
       <c r="K30" t="n">
         <v>0</v>
       </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -2104,10 +2034,8 @@
       <c r="K31" t="n">
         <v>540</v>
       </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>540</t>
-        </is>
+      <c r="L31" t="n">
+        <v>540</v>
       </c>
     </row>
     <row r="32">
@@ -2158,10 +2086,8 @@
       <c r="K32" t="n">
         <v>0</v>
       </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -2212,10 +2138,8 @@
       <c r="K33" t="n">
         <v>0</v>
       </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="L33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -2266,10 +2190,8 @@
       <c r="K34" t="n">
         <v>335</v>
       </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>335</t>
-        </is>
+      <c r="L34" t="n">
+        <v>335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>